<commit_message>
Case xlsx có parent kiểu số; ghi một đột biến tương đương
</commit_message>
<xml_diff>
--- a/conformance/cases/xlsx-04-numeric-ids.xlsx
+++ b/conformance/cases/xlsx-04-numeric-ids.xlsx
@@ -38,10 +38,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A</t>
-        </is>
+      <c r="A2">
+        <v>3</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -50,7 +48,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lane A</t>
+          <t xml:space="preserve">Lane số</t>
         </is>
       </c>
     </row>
@@ -63,10 +61,8 @@
           <t xml:space="preserve">start</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A</t>
-        </is>
+      <c r="C3">
+        <v>3</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -100,10 +96,8 @@
           <t xml:space="preserve">end</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A</t>
-        </is>
+      <c r="C5">
+        <v>3</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>

</xml_diff>